<commit_message>
list linh kien - ten gia tien cua TE8
</commit_message>
<xml_diff>
--- a/1. List linh kien/link_kien_mach.xlsx
+++ b/1. List linh kien/link_kien_mach.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2. Mr Tai\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2. Mr Tai\18. QN_Controller v1.1-20260920T050222Z-1-001\18. QN_Controller v1.1\2. PCB\PCB v1.1\1. List linh kien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1620C67-3A29-44ED-86FF-59428866A728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C04C498-0B9E-4246-B855-F88D268BA58A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,17 +18,26 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$F$1</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="51">
   <si>
     <t>STT</t>
   </si>
@@ -63,12 +72,6 @@
     <t>LED Xanh Lá 0805 Dán SMD Trong Suốt</t>
   </si>
   <si>
-    <t>5.240 đ</t>
-  </si>
-  <si>
-    <t>4.560 đ</t>
-  </si>
-  <si>
     <t>diode</t>
   </si>
   <si>
@@ -117,27 +120,9 @@
     <t>Tụ Nhôm SMD 100uF 50V 8x10.5mm</t>
   </si>
   <si>
-    <t>5.415 đ</t>
-  </si>
-  <si>
-    <t>2.622 đ</t>
-  </si>
-  <si>
-    <t>1.710 đ</t>
-  </si>
-  <si>
-    <t>9.959 đ</t>
-  </si>
-  <si>
-    <t>2.489 đ</t>
-  </si>
-  <si>
     <t>Điện Trở 0 Ohm 0805 5%</t>
   </si>
   <si>
-    <t>4.100 đ</t>
-  </si>
-  <si>
     <t>Điện Trở 330 Ohm 0805 5%</t>
   </si>
   <si>
@@ -162,9 +147,6 @@
     <t>2N7002 MOSFET Kênh N 60V 115mA SOT-23</t>
   </si>
   <si>
-    <t>9.120 đ</t>
-  </si>
-  <si>
     <t>Rơ le,relay</t>
   </si>
   <si>
@@ -174,27 +156,12 @@
     <t>BZT52C3V3 Diode Zener 3.3V 500mW</t>
   </si>
   <si>
-    <t>6.840 đ</t>
-  </si>
-  <si>
-    <t>4.560 đx2</t>
-  </si>
-  <si>
-    <t>15.000 đ</t>
-  </si>
-  <si>
     <t>https://shopee.vn/PC817-DIP-SOP-Opto-c%C3%A1ch-ly-quang-(-Combo-10-con-)-i.898903714.21577630595?extraParams=%7B%22display_model_id%22%3A98673463284%2C%22model_selection_logic%22%3A3%7D&amp;image_ids=vn-11134207-7ras8-m11gtjc69zq358</t>
   </si>
   <si>
     <t>Cuộn Cảm Dán SMD CD53 5852-101 100uH 4.5A</t>
   </si>
   <si>
-    <t>1.140 đ</t>
-  </si>
-  <si>
-    <t>18.368₫</t>
-  </si>
-  <si>
     <t>cuộn Cảm Điện Từ 1,5A 8x10mm 68uH</t>
   </si>
   <si>
@@ -204,58 +171,25 @@
     <t>https://shopee.vn/Combo-Relay-(R%E1%BB%9D-Le)-3V-5V-12V-24V-5-ch%C3%A2n-SongLe-i.684432731.23184799475?extraParams=%7B%22display_model_id%22%3A297798427357%2C%22model_selection_logic%22%3A3%7D&amp;image_ids=vn-11134201-81ztc-mud1poyzokchc1</t>
   </si>
   <si>
-    <t>8.499 đ</t>
-  </si>
-  <si>
-    <t>8.500 đ</t>
-  </si>
-  <si>
-    <t>60.192 đ</t>
-  </si>
-  <si>
-    <t>3.160 đ</t>
-  </si>
-  <si>
     <t>LM2596S-3.3 IC Điều Chỉnh Giảm Áp 3.3V 3A TO-263-5</t>
   </si>
   <si>
-    <t>10.260 đ</t>
-  </si>
-  <si>
     <t>https://shopee.vn/IC-3843-SOP-8-Ch%C3%A2n-D%C3%A1n-Ch%C3%ADnh-H%C3%A3ng-i.49512422.9989297527?extraParams=%7B%22display_model_id%22%3A94148027024%2C%22model_selection_logic%22%3A3%7D&amp;image_ids=sg-11134201-824in-mptmhcup02yq64</t>
   </si>
   <si>
-    <t>3.420 đ</t>
-  </si>
-  <si>
     <t>SR240 Diode Schottky 2A 40V</t>
   </si>
   <si>
-    <t>5.700 đ</t>
-  </si>
-  <si>
     <t>1N5822 Diode Schottky 40V 3A DO-201AD</t>
   </si>
   <si>
-    <t>6.270 đ</t>
-  </si>
-  <si>
     <t>SMAJ24CA TVS DIODE 24V 38.9V DO-214AC, SMA</t>
   </si>
   <si>
     <t>https://shopee.vn/(20-100-chi%E1%BA%BFc)-SMAJ24A-BZ-SMA-TVS-Diode-SMD-K%C3%AAnh-m%E1%BB%99t-h%C6%B0%E1%BB%9Bng-%C4%90i%E1%BB%91t-%C4%91i%E1%BB%87n-%C3%A1p-tho%C3%A1ng-qua-i.1834388203.45013841730?extraParams=%7B%22display_model_id%22%3A401194621797%2C%22model_selection_logic%22%3A3%7D&amp;image_ids=sg-11134201-8259b-mqj19ygjlo1s8c</t>
   </si>
   <si>
-    <t>17.505 đ</t>
-  </si>
-  <si>
     <t>1N5822</t>
-  </si>
-  <si>
-    <t>1.254 đ</t>
-  </si>
-  <si>
-    <t>6.830 đ*2</t>
   </si>
 </sst>
 </file>
@@ -287,18 +221,12 @@
       <name val="Roboto"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -313,13 +241,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -637,64 +564,64 @@
         <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D2" s="1">
         <v>20</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>49</v>
+      <c r="E2" s="1">
+        <v>4.5599999999999996</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="18">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D3" s="1">
         <v>5</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>29</v>
+      <c r="E3" s="1">
+        <v>5.415</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="18">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D4" s="1">
         <v>1</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>30</v>
+      <c r="E4" s="1">
+        <v>2.6219999999999999</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="18">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D5" s="1">
         <v>1</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>31</v>
+      <c r="E5" s="1">
+        <v>1.71</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="18">
@@ -708,11 +635,11 @@
       <c r="D6" s="1">
         <v>20</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>11</v>
+      <c r="E6" s="1">
+        <v>5.24</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="18">
@@ -726,401 +653,405 @@
       <c r="D7" s="1">
         <v>1</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>32</v>
+      <c r="E7" s="1">
+        <v>9.9589999999999996</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="18">
       <c r="A8" s="1"/>
       <c r="B8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="D8" s="1">
         <v>1</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>33</v>
+      <c r="E8" s="1">
+        <v>2.4889999999999999</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="18">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D9" s="1">
         <v>4</v>
       </c>
-      <c r="E9" s="1"/>
-      <c r="F9" s="3"/>
+      <c r="E9" s="1">
+        <v>20.52</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="10" spans="1:6" ht="18">
       <c r="B10" s="1"/>
       <c r="C10" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D10" s="1">
         <v>1</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>61</v>
+      <c r="E10" s="1">
+        <v>3.16</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="18">
       <c r="B11" s="1"/>
       <c r="C11" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D11" s="1">
         <v>1</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>60</v>
+      <c r="E11" s="1">
+        <v>60.192</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="18">
       <c r="B12" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="D12" s="1">
         <v>1</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>63</v>
+      <c r="E12" s="1">
+        <v>10.26</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="18">
       <c r="C13" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D13" s="1">
         <v>1</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>59</v>
+      <c r="E13" s="1">
+        <v>8.5</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="18">
       <c r="C14" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D14" s="1">
         <v>1</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>65</v>
+      <c r="E14" s="1">
+        <v>3.42</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="18">
       <c r="C15" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D15" s="1">
         <v>10</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>50</v>
+      <c r="E15" s="1">
+        <v>15</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="18">
       <c r="C16" s="1" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="D16" s="1">
         <v>5</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>69</v>
+      <c r="E16" s="1">
+        <v>6.27</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="2:6" ht="18">
       <c r="C17" s="1" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="D17" s="1">
         <v>50</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>35</v>
+      <c r="E17" s="1">
+        <v>4.0999999999999996</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="2:6" ht="18">
       <c r="C18" s="1" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="D18" s="1">
         <v>50</v>
       </c>
-      <c r="E18" s="1" t="s">
-        <v>35</v>
+      <c r="E18" s="1">
+        <v>4.0999999999999996</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="2:6" ht="18">
       <c r="C19" s="1" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="D19" s="1">
         <v>50</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>35</v>
+      <c r="E19" s="1">
+        <v>4.0999999999999996</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="2:6" ht="18">
       <c r="C20" s="1" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="D20" s="1">
         <v>50</v>
       </c>
-      <c r="E20" s="1" t="s">
-        <v>35</v>
+      <c r="E20" s="1">
+        <v>4.0999999999999996</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="2:6" ht="18">
       <c r="C21" s="1" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D21" s="1">
         <v>50</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>35</v>
+      <c r="E21" s="1">
+        <v>4.0999999999999996</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="2:6" ht="18">
       <c r="C22" s="1" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="D22" s="1">
         <v>50</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>35</v>
+      <c r="E22" s="1">
+        <v>4.0999999999999996</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="2:6" ht="18">
       <c r="C23" s="1" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="D23" s="1">
         <v>50</v>
       </c>
-      <c r="E23" s="1" t="s">
-        <v>35</v>
+      <c r="E23" s="1">
+        <v>4.0999999999999996</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="2:6" ht="18">
       <c r="C24" s="1" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D24" s="1">
-        <v>20</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>75</v>
+        <v>40</v>
+      </c>
+      <c r="E24" s="1">
+        <v>6.83</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="2:6" ht="18">
       <c r="C25" s="1" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="D25" s="1">
         <v>20</v>
       </c>
-      <c r="E25" s="1" t="s">
-        <v>44</v>
+      <c r="E25" s="1">
+        <v>9.1199999999999992</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="2:6" ht="18">
       <c r="C26" s="1" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="D26" s="1">
         <v>4</v>
       </c>
-      <c r="E26" s="1" t="s">
-        <v>58</v>
+      <c r="E26" s="1">
+        <v>8.4990000000000006</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27" spans="2:6" ht="18">
       <c r="B27" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D27" s="1">
         <v>1</v>
       </c>
-      <c r="E27" s="1" t="s">
-        <v>12</v>
+      <c r="E27" s="1">
+        <v>4.5599999999999996</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28" spans="2:6" ht="18">
       <c r="B28" s="1"/>
-      <c r="C28" s="4" t="s">
-        <v>73</v>
+      <c r="C28" s="3" t="s">
+        <v>50</v>
       </c>
       <c r="D28" s="1">
         <v>1</v>
       </c>
-      <c r="E28" s="1" t="s">
-        <v>74</v>
+      <c r="E28" s="1">
+        <v>1.254</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29" spans="2:6" ht="18">
       <c r="B29" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C29" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>66</v>
       </c>
       <c r="D29" s="1">
         <v>10</v>
       </c>
-      <c r="E29" s="1" t="s">
-        <v>67</v>
+      <c r="E29" s="1">
+        <v>5.7</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="30" spans="2:6" ht="18">
       <c r="C30" s="1" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="D30" s="1">
         <v>20</v>
       </c>
-      <c r="E30" s="1" t="s">
-        <v>48</v>
+      <c r="E30" s="1">
+        <v>6.84</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31" spans="2:6" ht="18">
       <c r="C31" s="1" t="s">
-        <v>70</v>
+        <v>48</v>
       </c>
       <c r="D31" s="1">
         <v>20</v>
       </c>
-      <c r="E31" s="1" t="s">
-        <v>72</v>
+      <c r="E31" s="1">
+        <v>17.504999999999999</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" spans="2:6" ht="18">
-      <c r="C32" s="5" t="s">
-        <v>52</v>
+      <c r="C32" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="D32" s="1">
         <v>1</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>53</v>
+      <c r="E32" s="1">
+        <v>1.1399999999999999</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="33" spans="3:6" ht="18">
-      <c r="C33" s="5" t="s">
-        <v>55</v>
+      <c r="C33" s="4" t="s">
+        <v>41</v>
       </c>
       <c r="D33" s="1">
         <v>1</v>
       </c>
-      <c r="E33" s="1" t="s">
-        <v>54</v>
+      <c r="E33" s="1">
+        <v>18.367999999999999</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
     </row>
     <row r="34" spans="3:6" ht="18">
-      <c r="C34" s="5"/>
+      <c r="C34" s="4"/>
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
     </row>
     <row r="35" spans="3:6" ht="18">
-      <c r="C35" s="5"/>
+      <c r="C35" s="4"/>
     </row>
     <row r="36" spans="3:6" ht="18">
-      <c r="C36" s="5"/>
+      <c r="C36" s="4"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>

</xml_diff>